<commit_message>
Add Job8Process, Job9 workflows, refine Bank page workflows (CloseCardPopup, SendMoney, GetMoney, FilterMypage etc.), update Main.xaml and Job6/Job8 processes
</commit_message>
<xml_diff>
--- a/Data/Input/Job8/send_money.xlsx
+++ b/Data/Input/Job8/send_money.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Documents\UiPath\Uipath_Study\Data\Input\Job8\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{872F281A-980F-434B-A083-9C819C6E1261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41035C09-A8F3-4758-94C7-677A8E098343}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38400" yWindow="1920" windowWidth="15240" windowHeight="12435" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -389,7 +389,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>240000</v>
+        <v>2315166</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
@@ -397,7 +397,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>3600000</v>
+        <v>1200000</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -405,7 +405,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>200000</v>
+        <v>256033</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>